<commit_message>
Daten einlesen überarbeiten, WIP
</commit_message>
<xml_diff>
--- a/w-daten-einlesen/folien/daten/tabelle.xlsx
+++ b/w-daten-einlesen/folien/daten/tabelle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11108"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maba/sciebo/mathematik-fbb/mathematik-b/02-folien-R/10-daten-lesen-und-aufbereiten/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maba/Documents/hs-bochum/40-projekte/bcd/bcd-bausteine-r/w-daten-einlesen/folien/daten/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90532C62-28B9-7140-92BA-223F78BDBF7F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8883E702-B279-C24A-838D-97BC538FB23C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5560" yWindow="460" windowWidth="28040" windowHeight="17040" xr2:uid="{9717EC76-56A2-B947-89AD-18FDA30351A2}"/>
+    <workbookView xWindow="3600" yWindow="2060" windowWidth="18800" windowHeight="11360" xr2:uid="{9717EC76-56A2-B947-89AD-18FDA30351A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy;@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -87,30 +87,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -125,28 +107,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -166,9 +145,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -206,7 +185,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -312,7 +291,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -454,7 +433,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -463,90 +442,100 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01105DAD-2E5C-D349-98E3-F059ED26C471}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>41273</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="7"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="D2" s="6"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>41274</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2">
         <v>30</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="7"/>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>41275</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="2">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>41276</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2">
         <v>50</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="7"/>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>41277</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="2">
         <v>2</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="7"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="2"/>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="4"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="4"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="4"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>